<commit_message>
Adaptando el script a todas las matrices, queda funcional, continuar con refactor de los modulos
</commit_message>
<xml_diff>
--- a/script/Config/Config.xlsx
+++ b/script/Config/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\25004549\Documents\02. UiPath Projects\00. M1\02. Certification_upcoming_expirations\notebook\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\25004549\Documents\02. UiPath Projects\00. M1\02. Certification_upcoming_expirations\notebook\script\Config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3249FD9E-1887-4ED8-9785-14FB54628431}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90C7C51E-F47B-4551-8722-7C60FB4F7FF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="53510" yWindow="-6320" windowWidth="10890" windowHeight="9550" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="53590" yWindow="2500" windowWidth="10720" windowHeight="9770" tabRatio="726" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Config" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="47">
   <si>
     <t>Sheet</t>
   </si>
@@ -46,9 +46,6 @@
     <t>Filename</t>
   </si>
   <si>
-    <t>Copy of 10.-SMD.xlsm</t>
-  </si>
-  <si>
     <t>Variable</t>
   </si>
   <si>
@@ -58,9 +55,6 @@
     <t>ShareFolder</t>
   </si>
   <si>
-    <t>C:\Users\25004549\Documents\02. UiPath Projects\00. M1\02. Certification_upcoming_expirations\notebook\data</t>
-  </si>
-  <si>
     <t>To</t>
   </si>
   <si>
@@ -73,22 +67,118 @@
     <t>ggaytan_itcj@hotmail.com</t>
   </si>
   <si>
-    <t>OP 1 C</t>
-  </si>
-  <si>
-    <t>OP 2 C</t>
-  </si>
-  <si>
-    <t>OP 3 C</t>
-  </si>
-  <si>
-    <t>OP 5 C</t>
-  </si>
-  <si>
-    <t>10.-SMT.xlsm</t>
-  </si>
-  <si>
-    <t>ggaytan.analytics@outlook.com</t>
+    <t>C:\Users\25004549\Documents\02. UiPath Projects\00. M1\02. Certification_upcoming_expirations\notebook\data\2026</t>
+  </si>
+  <si>
+    <t>Certificacciones PIR.xlsm</t>
+  </si>
+  <si>
+    <t>OPERADOR 1 CRITICO</t>
+  </si>
+  <si>
+    <t>OPERADOR 2</t>
+  </si>
+  <si>
+    <t>OPERADOR 3</t>
+  </si>
+  <si>
+    <t>OPERADOR 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Personal en areas nuevas </t>
+  </si>
+  <si>
+    <t>Certificacion GLASBREAK.xlsm</t>
+  </si>
+  <si>
+    <t>OP.CRITICO 1</t>
+  </si>
+  <si>
+    <t>OP.CRITICO 2</t>
+  </si>
+  <si>
+    <t>OP.CRITICO 5</t>
+  </si>
+  <si>
+    <t>Certificaciones  GRIP.xlsx</t>
+  </si>
+  <si>
+    <t>CRITICO.1</t>
+  </si>
+  <si>
+    <t>CRITICO.2</t>
+  </si>
+  <si>
+    <t>CRITICO.3</t>
+  </si>
+  <si>
+    <t>CRITICO.5</t>
+  </si>
+  <si>
+    <t>Certificaciones  SMD.xlsx</t>
+  </si>
+  <si>
+    <t>CRITICO 1</t>
+  </si>
+  <si>
+    <t>Certificaciones ATP.xlsx</t>
+  </si>
+  <si>
+    <t>CRITICO 2</t>
+  </si>
+  <si>
+    <t>CRITICO 3</t>
+  </si>
+  <si>
+    <t>CRITICO 5</t>
+  </si>
+  <si>
+    <t>Certificaciones GABINETES.xlsx</t>
+  </si>
+  <si>
+    <t>Certificaciones KEYPAD.xlsm</t>
+  </si>
+  <si>
+    <t>Certificaciones RADIO.xlsx</t>
+  </si>
+  <si>
+    <t>Certificaciones SLOAN.xlsx</t>
+  </si>
+  <si>
+    <t>certificados rts.xlsx</t>
+  </si>
+  <si>
+    <t>CONTACTOS.xlsm</t>
+  </si>
+  <si>
+    <t>SLOAN 4TO TURNO.xlsm</t>
+  </si>
+  <si>
+    <t>OP.CRITICO 3</t>
+  </si>
+  <si>
+    <t>Op#1</t>
+  </si>
+  <si>
+    <t>OP#2</t>
+  </si>
+  <si>
+    <t>HOJA 1  (3)</t>
+  </si>
+  <si>
+    <t>HOJA 1  (4)</t>
+  </si>
+  <si>
+    <t>HOJA 1  (5)</t>
+  </si>
+  <si>
+    <t>OP#3</t>
+  </si>
+  <si>
+    <t>OP#4</t>
+  </si>
+  <si>
+    <t>OP#5</t>
   </si>
 </sst>
 </file>
@@ -410,23 +500,23 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="98.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="103.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
         <v>3</v>
-      </c>
-      <c r="B1" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -436,11 +526,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B51"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
@@ -453,7 +543,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
         <v>11</v>
@@ -461,7 +551,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
         <v>12</v>
@@ -469,7 +559,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="B4" t="s">
         <v>13</v>
@@ -477,7 +567,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
         <v>14</v>
@@ -485,34 +575,370 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
         <v>15</v>
-      </c>
-      <c r="B6" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B8" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>14</v>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>25</v>
+      </c>
+      <c r="B16" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>27</v>
+      </c>
+      <c r="B21" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>31</v>
+      </c>
+      <c r="B22" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>31</v>
+      </c>
+      <c r="B23" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>31</v>
+      </c>
+      <c r="B24" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>31</v>
+      </c>
+      <c r="B25" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>32</v>
+      </c>
+      <c r="B26" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>32</v>
+      </c>
+      <c r="B27" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>32</v>
+      </c>
+      <c r="B28" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>32</v>
+      </c>
+      <c r="B29" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>33</v>
+      </c>
+      <c r="B30" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>33</v>
+      </c>
+      <c r="B32" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>33</v>
+      </c>
+      <c r="B33" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>34</v>
+      </c>
+      <c r="B34" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>34</v>
+      </c>
+      <c r="B35" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>34</v>
+      </c>
+      <c r="B36" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>34</v>
+      </c>
+      <c r="B37" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>35</v>
+      </c>
+      <c r="B38" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>35</v>
+      </c>
+      <c r="B39" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>35</v>
+      </c>
+      <c r="B40" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>35</v>
+      </c>
+      <c r="B41" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>36</v>
+      </c>
+      <c r="B42" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>36</v>
+      </c>
+      <c r="B43" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>36</v>
+      </c>
+      <c r="B44" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>36</v>
+      </c>
+      <c r="B45" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>36</v>
+      </c>
+      <c r="B46" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>37</v>
+      </c>
+      <c r="B47" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>37</v>
+      </c>
+      <c r="B48" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>37</v>
+      </c>
+      <c r="B49" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>37</v>
+      </c>
+      <c r="B50" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>37</v>
+      </c>
+      <c r="B51" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -522,7 +948,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DE519E4-A818-4069-9FBD-178C27634827}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="27.6328125" bestFit="1" customWidth="1"/>
@@ -531,23 +957,18 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>